<commit_message>
Update controls Gantt schedule
Refresh the Baja SAE controls project Gantt chart to reflect the current planning and milestone timeline for the controls work. This update keeps the schedule aligned with the project’s current development plan and priorities.
</commit_message>
<xml_diff>
--- a/Baja_SAE_Controls_Gantt.xlsx
+++ b/Baja_SAE_Controls_Gantt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexmiller/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB1571BD-393E-7344-AAC8-7CA4B8C36F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0FCC49-58C5-E54C-94F2-5BF7C9EA5D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="200">
   <si>
     <t>Baja SAE – Controls  |  Capstone Project Gantt Chart</t>
   </si>
@@ -659,6 +659,9 @@
   </si>
   <si>
     <t>Part Selection Deadline</t>
+  </si>
+  <si>
+    <t>AdI04</t>
   </si>
 </sst>
 </file>
@@ -6833,8 +6836,12 @@
       </c>
     </row>
     <row r="42" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="26"/>
-      <c r="B42" s="27"/>
+      <c r="A42" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="B42" s="27" t="s">
+        <v>197</v>
+      </c>
       <c r="C42" s="28" t="s">
         <v>198</v>
       </c>
@@ -6994,7 +7001,7 @@
     </row>
     <row r="43" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="26" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B43" s="27" t="s">
         <v>197</v>

</xml_diff>